<commit_message>
auditoria: adendo 4 — junho e julho eram um mes so, nao duplicata
Registra o que o commit anterior perdeu (crases viraram substituicao de comando
no shell): a causa e o dCompet do ADN vir com a data de emissao; as colunas sao
competencia_origem_adn e cancelamento_solicitado_em.

Inclui a licao: o sinal de que eu estava errado veio de graca e quase passou —
ao marcar as notas como canceladas o buraco de 100 mil nao fechou, ANDOU de mes.
Duplicata some; competencia trocada muda de lugar.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/auditoria/planilhas/lacunas_financeiro_20260813.xlsx
+++ b/auditoria/planilhas/lacunas_financeiro_20260813.xlsx
@@ -529,7 +529,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Duas notas do mesmo serviço, uma por CNPJ. Decidir qual vale. Sem isso o faturamento de julho fica R$108 mil acima do real.</t>
+          <t>Duas notas do mesmo CNPJ, mesmo cliente e mesmo valor dentro de julho. Confirmar se são dois serviços mesmo.</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -654,14 +654,14 @@
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>Julho fechou R$378.286,98 — R$108.386,92 acima dos outros meses. São pares do MESMO serviço faturados pelos DOIS CNPJs na transição. Nenhuma está cancelada no Ambiente Nacional, e o cliente pagou uma vez só. Marque qual vale; eu NÃO cancelo nota — cancelamento é ato fiscal e vai com o contador.</t>
+          <t>O degrau de R$108.386,92 em julho já foi resolvido: n109 e n111 são o faturamento de JUNHO, emitido pela Eletrônica em 09/07 e 14/07 — competência corrigida no sistema, junho voltou para R$271.916,59 e julho para R$269.900,06. Sobrou este par: duas notas do MESMO CNPJ, mesmo cliente e mesmo valor dentro de julho.</t>
         </is>
       </c>
     </row>
@@ -693,19 +693,19 @@
       </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
-          <t>Esta nota VALE? (sim/não)</t>
+          <t>São dois serviços mesmo? (sim/não)</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>Se não: cancelar ou já cancelada?</t>
+          <t>Se não: qual cancelar?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t>111</t>
+          <t>112</t>
         </is>
       </c>
       <c r="B4" s="9" t="inlineStr">
@@ -715,16 +715,16 @@
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>15/07/2026</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>CONDOMINIO IDEAL FLORES DA CIDADE</t>
+          <t>CONDOMINIO PARQUE RESIDENCIAL GELAIN</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
-        <v>65842.42</v>
+        <v>6000</v>
       </c>
       <c r="F4" s="9" t="n"/>
       <c r="G4" s="9" t="n"/>
@@ -732,137 +732,29 @@
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>115</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Conecta Mais Patrimonial</t>
+          <t>Conecta Mais Eletrônica</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>31/07/2026</t>
+          <t>29/07/2026</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>CONDOMINIO IDEAL FLORES DA CIDADE</t>
+          <t>CONDOMINIO PARQUE RESIDENCIAL GELAIN</t>
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>65842.42</v>
+        <v>6000</v>
       </c>
       <c r="F5" s="11" t="n"/>
       <c r="G5" s="11" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="inlineStr">
-        <is>
-          <t>Conecta Mais Eletrônica</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>15/07/2026</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>CONDOMINIO PARQUE RESIDENCIAL GELAIN</t>
-        </is>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F6" s="9" t="n"/>
-      <c r="G6" s="9" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
-      </c>
-      <c r="B7" s="11" t="inlineStr">
-        <is>
-          <t>Conecta Mais Eletrônica</t>
-        </is>
-      </c>
-      <c r="C7" s="11" t="inlineStr">
-        <is>
-          <t>29/07/2026</t>
-        </is>
-      </c>
-      <c r="D7" s="11" t="inlineStr">
-        <is>
-          <t>CONDOMINIO PARQUE RESIDENCIAL GELAIN</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>6000</v>
-      </c>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="11" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>109</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>Conecta Mais Eletrônica</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>09/07/2026</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>RESIDENCIAL LARANJEIRAS VILLAGE</t>
-        </is>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>42544.5</v>
-      </c>
-      <c r="F8" s="9" t="n"/>
-      <c r="G8" s="9" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>13</t>
-        </is>
-      </c>
-      <c r="B9" s="11" t="inlineStr">
-        <is>
-          <t>Conecta Mais Patrimonial</t>
-        </is>
-      </c>
-      <c r="C9" s="11" t="inlineStr">
-        <is>
-          <t>24/07/2026</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>RESIDENCIAL LARANJEIRAS VILLAGE</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>42544.5</v>
-      </c>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>